<commit_message>
feat: add URL styling rule and rename WAVE method to WAVES in StyleRegistry
</commit_message>
<xml_diff>
--- a/docs/Latency per message(tick).xlsx
+++ b/docs/Latency per message(tick).xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish-chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68DA3B0F-4C66-40B6-B1E0-47ACA2802F3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B544693-EA54-4997-998F-3D90F6E6C5ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
   <sheets>
-    <sheet name="v2.4.0" sheetId="5" r:id="rId1"/>
-    <sheet name="v2.3.0" sheetId="4" r:id="rId2"/>
-    <sheet name="v2.2.0" sheetId="1" r:id="rId3"/>
-    <sheet name="v2.1.0" sheetId="2" r:id="rId4"/>
-    <sheet name="v2.0.0" sheetId="3" r:id="rId5"/>
+    <sheet name="v2.5.1" sheetId="6" r:id="rId1"/>
+    <sheet name="v2.4.0" sheetId="5" r:id="rId2"/>
+    <sheet name="v2.3.0" sheetId="4" r:id="rId3"/>
+    <sheet name="v2.2.0" sheetId="1" r:id="rId4"/>
+    <sheet name="v2.1.0" sheetId="2" r:id="rId5"/>
+    <sheet name="v2.0.0" sheetId="3" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="24">
   <si>
     <t>Message Count/tick</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -512,6 +513,133 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80B5C1B6-EB74-483F-9F2C-AFF00761E6BD}">
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="2" width="14.8984375" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" customWidth="1"/>
+    <col min="4" max="4" width="20.5" customWidth="1"/>
+    <col min="5" max="5" width="16.69921875" customWidth="1"/>
+    <col min="6" max="6" width="16.796875" customWidth="1"/>
+    <col min="7" max="7" width="18.296875" customWidth="1"/>
+    <col min="8" max="8" width="16.59765625" customWidth="1"/>
+    <col min="9" max="9" width="28.09765625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A3">
+        <v>50</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A4">
+        <v>100</v>
+      </c>
+      <c r="B4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A5">
+        <v>200</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A6">
+        <v>300</v>
+      </c>
+      <c r="B6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A7">
+        <v>400</v>
+      </c>
+      <c r="B7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="A8">
+        <v>500</v>
+      </c>
+      <c r="B8">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06116B37-F902-49E7-B259-88C657E3068D}">
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -765,7 +893,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F548A5A-373E-4879-9567-B3774331AE70}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1060,7 +1188,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B38E37E-D8A4-4D05-B5EE-C32E8023EE69}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1355,7 +1483,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63723110-D812-4C3D-AFC0-E7634718A855}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1514,7 +1642,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0A4C8FE-4793-4DF4-BD4A-84084E113CBB}">
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>

</xml_diff>

<commit_message>
docs: update README with version change to 2.5.1 and mention latency analysis details
</commit_message>
<xml_diff>
--- a/docs/Latency per message(tick).xlsx
+++ b/docs/Latency per message(tick).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish-chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B544693-EA54-4997-998F-3D90F6E6C5ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E978681-5275-4496-B13D-D7DBDDFE4C70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
   <sheets>
     <sheet name="v2.5.1" sheetId="6" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
   <si>
     <t>Message Count/tick</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -130,6 +130,22 @@
   </si>
   <si>
     <t>200char/Mixed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>50char/Mention Only(notification off)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>50char/Mention Only(notification on)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>200char/Mention Only(notification off)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>200char/Mention Only(notification on)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -514,20 +530,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80B5C1B6-EB74-483F-9F2C-AFF00761E6BD}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="2" width="14.8984375" customWidth="1"/>
     <col min="3" max="3" width="19.59765625" customWidth="1"/>
-    <col min="4" max="4" width="20.5" customWidth="1"/>
-    <col min="5" max="5" width="16.69921875" customWidth="1"/>
-    <col min="6" max="6" width="16.796875" customWidth="1"/>
+    <col min="4" max="4" width="33.796875" customWidth="1"/>
+    <col min="5" max="5" width="31.296875" customWidth="1"/>
+    <col min="6" max="6" width="13.8984375" customWidth="1"/>
     <col min="7" max="7" width="18.296875" customWidth="1"/>
-    <col min="8" max="8" width="16.59765625" customWidth="1"/>
-    <col min="9" max="9" width="28.09765625" customWidth="1"/>
+    <col min="8" max="8" width="18.19921875" customWidth="1"/>
+    <col min="9" max="9" width="31.59765625" customWidth="1"/>
+    <col min="10" max="10" width="20.09765625" customWidth="1"/>
+    <col min="11" max="11" width="12.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -538,25 +556,31 @@
         <v>17</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="E1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" t="s">
         <v>19</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>20</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>21</v>
       </c>
-      <c r="H1" t="s">
-        <v>22</v>
-      </c>
       <c r="I1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>0</v>
       </c>
@@ -584,8 +608,11 @@
       <c r="I2">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
+      <c r="J2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>50</v>
       </c>
@@ -593,7 +620,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>100</v>
       </c>
@@ -601,7 +628,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>200</v>
       </c>
@@ -609,7 +636,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>300</v>
       </c>
@@ -617,7 +644,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>400</v>
       </c>
@@ -625,7 +652,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>500</v>
       </c>

</xml_diff>

<commit_message>
docs: update README to clarify mention types and performance metrics terminology
</commit_message>
<xml_diff>
--- a/docs/Latency per message(tick).xlsx
+++ b/docs/Latency per message(tick).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish-chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E978681-5275-4496-B13D-D7DBDDFE4C70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F0C530-4CA2-4F07-87E4-16088270D7D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
@@ -530,10 +530,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80B5C1B6-EB74-483F-9F2C-AFF00761E6BD}">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="2" width="14.8984375" customWidth="1"/>
+    <col min="1" max="1" width="14.8984375" customWidth="1"/>
+    <col min="2" max="2" width="17.19921875" customWidth="1"/>
     <col min="3" max="3" width="19.59765625" customWidth="1"/>
     <col min="4" max="4" width="33.796875" customWidth="1"/>
     <col min="5" max="5" width="31.296875" customWidth="1"/>
@@ -541,8 +542,8 @@
     <col min="7" max="7" width="18.296875" customWidth="1"/>
     <col min="8" max="8" width="18.19921875" customWidth="1"/>
     <col min="9" max="9" width="31.59765625" customWidth="1"/>
-    <col min="10" max="10" width="20.09765625" customWidth="1"/>
-    <col min="11" max="11" width="12.5" customWidth="1"/>
+    <col min="10" max="10" width="33.69921875" customWidth="1"/>
+    <col min="11" max="11" width="18.19921875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.4">
@@ -630,33 +631,17 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A5">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A6">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="B6">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A7">
-        <v>400</v>
-      </c>
-      <c r="B7">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.4">
-      <c r="A8">
-        <v>500</v>
-      </c>
-      <c r="B8">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: update README.md for version 2.6.0 with new image links and references
</commit_message>
<xml_diff>
--- a/docs/Latency per message(tick).xlsx
+++ b/docs/Latency per message(tick).xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish-chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F0C530-4CA2-4F07-87E4-16088270D7D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EE85E6E-ED46-4D86-9288-0D9A8A1592B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
   <sheets>
-    <sheet name="v2.5.1" sheetId="6" r:id="rId1"/>
+    <sheet name="v2.6.0" sheetId="6" r:id="rId1"/>
     <sheet name="v2.4.0" sheetId="5" r:id="rId2"/>
     <sheet name="v2.3.0" sheetId="4" r:id="rId3"/>
     <sheet name="v2.2.0" sheetId="1" r:id="rId4"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="34">
   <si>
     <t>Message Count/tick</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -133,20 +133,34 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>50char/Plain Text</t>
+  </si>
+  <si>
+    <t>50char/Styling Only</t>
+  </si>
+  <si>
+    <t>50char/Mention Only(notification on)</t>
+  </si>
+  <si>
     <t>50char/Mention Only(notification off)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>50char/Mention Only(notification on)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>50char/Mixed</t>
+  </si>
+  <si>
+    <t>200char/Plain Text</t>
+  </si>
+  <si>
+    <t>200char/Styling Only</t>
+  </si>
+  <si>
+    <t>200char/Mention Only(notification on)</t>
   </si>
   <si>
     <t>200char/Mention Only(notification off)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>200char/Mention Only(notification on)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>200char/Mixed</t>
   </si>
 </sst>
 </file>
@@ -548,37 +562,37 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C1" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F1" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="G1" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="H1" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="I1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="J1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="K1" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.4">
@@ -612,13 +626,43 @@
       <c r="J2">
         <v>2</v>
       </c>
+      <c r="K2">
+        <v>2</v>
+      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>50</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>6</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3">
+        <v>12</v>
+      </c>
+      <c r="J3">
+        <v>8</v>
+      </c>
+      <c r="K3">
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.4">
@@ -628,6 +672,33 @@
       <c r="B4">
         <v>4</v>
       </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4">
+        <v>8</v>
+      </c>
+      <c r="E4">
+        <v>6</v>
+      </c>
+      <c r="F4">
+        <v>5</v>
+      </c>
+      <c r="G4">
+        <v>5</v>
+      </c>
+      <c r="H4">
+        <v>7</v>
+      </c>
+      <c r="I4">
+        <v>18</v>
+      </c>
+      <c r="J4">
+        <v>14</v>
+      </c>
+      <c r="K4">
+        <v>10</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A5">
@@ -636,6 +707,33 @@
       <c r="B5">
         <v>6</v>
       </c>
+      <c r="C5">
+        <v>9</v>
+      </c>
+      <c r="D5">
+        <v>13</v>
+      </c>
+      <c r="E5">
+        <v>11</v>
+      </c>
+      <c r="F5">
+        <v>12</v>
+      </c>
+      <c r="G5">
+        <v>9</v>
+      </c>
+      <c r="H5">
+        <v>14</v>
+      </c>
+      <c r="I5">
+        <v>32</v>
+      </c>
+      <c r="J5">
+        <v>26</v>
+      </c>
+      <c r="K5">
+        <v>18</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A6">
@@ -643,6 +741,33 @@
       </c>
       <c r="B6">
         <v>8</v>
+      </c>
+      <c r="C6">
+        <v>12</v>
+      </c>
+      <c r="D6">
+        <v>19</v>
+      </c>
+      <c r="E6">
+        <v>15</v>
+      </c>
+      <c r="F6">
+        <v>16</v>
+      </c>
+      <c r="G6">
+        <v>14</v>
+      </c>
+      <c r="H6">
+        <v>19</v>
+      </c>
+      <c r="I6">
+        <v>55</v>
+      </c>
+      <c r="J6">
+        <v>35</v>
+      </c>
+      <c r="K6">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: ensure options are retrieved correctly when presets are blank
</commit_message>
<xml_diff>
--- a/docs/Latency per message(tick).xlsx
+++ b/docs/Latency per message(tick).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish-chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EE85E6E-ED46-4D86-9288-0D9A8A1592B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2584E54B-3AB8-449A-8B93-D46395187918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
@@ -761,7 +761,7 @@
         <v>19</v>
       </c>
       <c r="I6">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J6">
         <v>35</v>

</xml_diff>

<commit_message>
fix: update version numbers and image links in README for v2.6.1
</commit_message>
<xml_diff>
--- a/docs/Latency per message(tick).xlsx
+++ b/docs/Latency per message(tick).xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish-chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2584E54B-3AB8-449A-8B93-D46395187918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0E6ED2-CFED-4B9A-B35B-E03351889ECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
   <sheets>
-    <sheet name="v2.6.0" sheetId="6" r:id="rId1"/>
-    <sheet name="v2.4.0" sheetId="5" r:id="rId2"/>
-    <sheet name="v2.3.0" sheetId="4" r:id="rId3"/>
-    <sheet name="v2.2.0" sheetId="1" r:id="rId4"/>
-    <sheet name="v2.1.0" sheetId="2" r:id="rId5"/>
-    <sheet name="v2.0.0" sheetId="3" r:id="rId6"/>
+    <sheet name="v2.6.1" sheetId="7" r:id="rId1"/>
+    <sheet name="v2.6.0" sheetId="6" r:id="rId2"/>
+    <sheet name="v2.4.0" sheetId="5" r:id="rId3"/>
+    <sheet name="v2.3.0" sheetId="4" r:id="rId4"/>
+    <sheet name="v2.2.0" sheetId="1" r:id="rId5"/>
+    <sheet name="v2.1.0" sheetId="2" r:id="rId6"/>
+    <sheet name="v2.0.0" sheetId="3" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="34">
   <si>
     <t>Message Count/tick</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -543,6 +544,240 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D97B426B-7A31-4528-9C0B-EA092DD19299}">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="14.8984375" customWidth="1"/>
+    <col min="2" max="2" width="17.19921875" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" customWidth="1"/>
+    <col min="4" max="4" width="33.796875" customWidth="1"/>
+    <col min="5" max="5" width="31.296875" customWidth="1"/>
+    <col min="6" max="6" width="13.8984375" customWidth="1"/>
+    <col min="7" max="7" width="18.296875" customWidth="1"/>
+    <col min="8" max="8" width="18.19921875" customWidth="1"/>
+    <col min="9" max="9" width="31.59765625" customWidth="1"/>
+    <col min="10" max="10" width="33.69921875" customWidth="1"/>
+    <col min="11" max="11" width="18.19921875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" t="s">
+        <v>31</v>
+      </c>
+      <c r="J1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A3">
+        <v>50</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>5</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>4</v>
+      </c>
+      <c r="I3">
+        <v>8</v>
+      </c>
+      <c r="J3">
+        <v>7</v>
+      </c>
+      <c r="K3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A4">
+        <v>100</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>8</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4">
+        <v>4</v>
+      </c>
+      <c r="G4">
+        <v>5</v>
+      </c>
+      <c r="H4">
+        <v>8</v>
+      </c>
+      <c r="I4">
+        <v>14</v>
+      </c>
+      <c r="J4">
+        <v>10</v>
+      </c>
+      <c r="K4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A5">
+        <v>300</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>9</v>
+      </c>
+      <c r="D5">
+        <v>13</v>
+      </c>
+      <c r="E5">
+        <v>10</v>
+      </c>
+      <c r="F5">
+        <v>11</v>
+      </c>
+      <c r="G5">
+        <v>9</v>
+      </c>
+      <c r="H5">
+        <v>15</v>
+      </c>
+      <c r="I5">
+        <v>30</v>
+      </c>
+      <c r="J5">
+        <v>23</v>
+      </c>
+      <c r="K5">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A6">
+        <v>500</v>
+      </c>
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>12</v>
+      </c>
+      <c r="D6">
+        <v>18</v>
+      </c>
+      <c r="E6">
+        <v>14</v>
+      </c>
+      <c r="F6">
+        <v>15</v>
+      </c>
+      <c r="G6">
+        <v>13</v>
+      </c>
+      <c r="H6">
+        <v>19</v>
+      </c>
+      <c r="I6">
+        <v>48</v>
+      </c>
+      <c r="J6">
+        <v>32</v>
+      </c>
+      <c r="K6">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80B5C1B6-EB74-483F-9F2C-AFF00761E6BD}">
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -776,7 +1011,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06116B37-F902-49E7-B259-88C657E3068D}">
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1030,7 +1265,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F548A5A-373E-4879-9567-B3774331AE70}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1325,7 +1560,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B38E37E-D8A4-4D05-B5EE-C32E8023EE69}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1620,7 +1855,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63723110-D812-4C3D-AFC0-E7634718A855}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1779,7 +2014,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0A4C8FE-4793-4DF4-BD4A-84084E113CBB}">
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>

</xml_diff>

<commit_message>
fix: update image links and version references in documentation
</commit_message>
<xml_diff>
--- a/docs/Latency per message(tick).xlsx
+++ b/docs/Latency per message(tick).xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whghk\Desktop\Coding\Intellij\embellish-chat\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0E6ED2-CFED-4B9A-B35B-E03351889ECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73DBC064-CC80-4D4C-A46A-F84D2D3ED81F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{30AE5353-CC8E-4A31-864B-BE4B1A53EFC5}"/>
   </bookViews>
   <sheets>
-    <sheet name="v2.6.1" sheetId="7" r:id="rId1"/>
-    <sheet name="v2.6.0" sheetId="6" r:id="rId2"/>
-    <sheet name="v2.4.0" sheetId="5" r:id="rId3"/>
-    <sheet name="v2.3.0" sheetId="4" r:id="rId4"/>
-    <sheet name="v2.2.0" sheetId="1" r:id="rId5"/>
-    <sheet name="v2.1.0" sheetId="2" r:id="rId6"/>
-    <sheet name="v2.0.0" sheetId="3" r:id="rId7"/>
+    <sheet name="3.0.0" sheetId="8" r:id="rId1"/>
+    <sheet name="v2.6.1" sheetId="7" r:id="rId2"/>
+    <sheet name="v2.6.0" sheetId="6" r:id="rId3"/>
+    <sheet name="v2.4.0" sheetId="5" r:id="rId4"/>
+    <sheet name="v2.3.0" sheetId="4" r:id="rId5"/>
+    <sheet name="v2.2.0" sheetId="1" r:id="rId6"/>
+    <sheet name="v2.1.0" sheetId="2" r:id="rId7"/>
+    <sheet name="v2.0.0" sheetId="3" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="34">
   <si>
     <t>Message Count/tick</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -544,6 +545,240 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E78EE54-DA90-4103-8C68-FDEA76202166}">
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="18.296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.69921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.19921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.69921875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.69921875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.8984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="34.296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="34.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.796875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" t="s">
+        <v>31</v>
+      </c>
+      <c r="J1" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A3">
+        <v>50</v>
+      </c>
+      <c r="B3">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <v>4</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3">
+        <v>7</v>
+      </c>
+      <c r="J3">
+        <v>7</v>
+      </c>
+      <c r="K3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A4">
+        <v>100</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4">
+        <v>5</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4">
+        <v>5</v>
+      </c>
+      <c r="G4">
+        <v>5</v>
+      </c>
+      <c r="H4">
+        <v>7</v>
+      </c>
+      <c r="I4">
+        <v>11</v>
+      </c>
+      <c r="J4">
+        <v>9</v>
+      </c>
+      <c r="K4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A5">
+        <v>300</v>
+      </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <v>9</v>
+      </c>
+      <c r="D5">
+        <v>10</v>
+      </c>
+      <c r="E5">
+        <v>10</v>
+      </c>
+      <c r="F5">
+        <v>11</v>
+      </c>
+      <c r="G5">
+        <v>11</v>
+      </c>
+      <c r="H5">
+        <v>14</v>
+      </c>
+      <c r="I5">
+        <v>23</v>
+      </c>
+      <c r="J5">
+        <v>21</v>
+      </c>
+      <c r="K5">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
+      <c r="A6">
+        <v>500</v>
+      </c>
+      <c r="B6">
+        <v>8</v>
+      </c>
+      <c r="C6">
+        <v>11</v>
+      </c>
+      <c r="D6">
+        <v>14</v>
+      </c>
+      <c r="E6">
+        <v>14</v>
+      </c>
+      <c r="F6">
+        <v>14</v>
+      </c>
+      <c r="G6">
+        <v>14</v>
+      </c>
+      <c r="H6">
+        <v>18</v>
+      </c>
+      <c r="I6">
+        <v>34</v>
+      </c>
+      <c r="J6">
+        <v>31</v>
+      </c>
+      <c r="K6">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D97B426B-7A31-4528-9C0B-EA092DD19299}">
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -642,7 +877,7 @@
         <v>4</v>
       </c>
       <c r="D3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -677,7 +912,7 @@
         <v>5</v>
       </c>
       <c r="D4">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E4">
         <v>5</v>
@@ -712,7 +947,7 @@
         <v>9</v>
       </c>
       <c r="D5">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="E5">
         <v>10</v>
@@ -747,7 +982,7 @@
         <v>12</v>
       </c>
       <c r="D6">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E6">
         <v>14</v>
@@ -777,7 +1012,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80B5C1B6-EB74-483F-9F2C-AFF00761E6BD}">
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1011,7 +1246,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06116B37-F902-49E7-B259-88C657E3068D}">
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1265,7 +1500,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F548A5A-373E-4879-9567-B3774331AE70}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1560,7 +1795,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B38E37E-D8A4-4D05-B5EE-C32E8023EE69}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -1855,7 +2090,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63723110-D812-4C3D-AFC0-E7634718A855}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
@@ -2014,7 +2249,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0A4C8FE-4793-4DF4-BD4A-84084E113CBB}">
   <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>

</xml_diff>